<commit_message>
Professional polish: DOCX/XLSX content refined
</commit_message>
<xml_diff>
--- a/pack/AI-Systems-Register.xlsx
+++ b/pack/AI-Systems-Register.xlsx
@@ -28,6 +28,7 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -39,12 +40,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000066CC"/>
-        <bgColor rgb="000066CC"/>
+        <fgColor rgb="00012060"/>
+        <bgColor rgb="00012060"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,14 +53,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,23 +433,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tool Name</t>
+          <t>Tool</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -457,12 +465,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Data Access Level</t>
+          <t>Data Access</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Risk Level</t>
+          <t>Risk</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -478,6 +486,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -499,17 +512,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>[Approver]</t>
+          <t>[Name]</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -522,6 +535,7 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -541,7 +555,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Internal</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -551,7 +565,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[Approver]</t>
+          <t>[Name]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -564,6 +578,7 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -583,17 +598,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>Internal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>[Approver]</t>
+          <t>[Name]</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -606,6 +621,7 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>